<commit_message>
docs: finalize FINNest Day 1 requirements and V1 scope
</commit_message>
<xml_diff>
--- a/tracking/Project_Checklist.xlsx
+++ b/tracking/Project_Checklist.xlsx
@@ -28,7 +28,7 @@
     <t>Verified V1 features</t>
   </si>
   <si>
-    <t>0 / 144</t>
+    <t>0 / 140</t>
   </si>
   <si>
     <t>V1 feature progress</t>
@@ -382,6 +382,9 @@
     <t>FIN-027</t>
   </si>
   <si>
+    <t>V1.5</t>
+  </si>
+  <si>
     <t>Supported bank PDF parser #2</t>
   </si>
   <si>
@@ -1469,9 +1472,6 @@
   </si>
   <si>
     <t>FIN-145</t>
-  </si>
-  <si>
-    <t>V1.5</t>
   </si>
   <si>
     <t>Expanded personal finance</t>
@@ -4134,20 +4134,18 @@
         <v>121</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>28</v>
+        <v>122</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>91</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="G31" s="8">
-        <v>14</v>
-      </c>
+      <c r="G31" s="8"/>
       <c r="H31" s="8" t="s">
         <v>32</v>
       </c>
@@ -4166,7 +4164,7 @@
         <v>26</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>28</v>
@@ -4175,7 +4173,7 @@
         <v>91</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F32" s="11" t="s">
         <v>31</v>
@@ -4187,7 +4185,7 @@
         <v>32</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J32" s="11" t="s">
         <v>34</v>
@@ -4201,7 +4199,7 @@
         <v>26</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>28</v>
@@ -4210,7 +4208,7 @@
         <v>91</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>31</v>
@@ -4222,7 +4220,7 @@
         <v>32</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J33" s="8" t="s">
         <v>34</v>
@@ -4236,7 +4234,7 @@
         <v>26</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>28</v>
@@ -4245,7 +4243,7 @@
         <v>91</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F34" s="11" t="s">
         <v>31</v>
@@ -4257,7 +4255,7 @@
         <v>32</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J34" s="11" t="s">
         <v>34</v>
@@ -4271,7 +4269,7 @@
         <v>26</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>28</v>
@@ -4280,7 +4278,7 @@
         <v>91</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F35" s="8" t="s">
         <v>31</v>
@@ -4292,7 +4290,7 @@
         <v>32</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J35" s="8" t="s">
         <v>34</v>
@@ -4306,7 +4304,7 @@
         <v>26</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>28</v>
@@ -4315,7 +4313,7 @@
         <v>91</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F36" s="11" t="s">
         <v>31</v>
@@ -4327,7 +4325,7 @@
         <v>32</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J36" s="11" t="s">
         <v>34</v>
@@ -4341,7 +4339,7 @@
         <v>26</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>28</v>
@@ -4350,7 +4348,7 @@
         <v>91</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>31</v>
@@ -4362,7 +4360,7 @@
         <v>32</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>34</v>
@@ -4376,7 +4374,7 @@
         <v>26</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>28</v>
@@ -4385,7 +4383,7 @@
         <v>91</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F38" s="11" t="s">
         <v>31</v>
@@ -4397,7 +4395,7 @@
         <v>32</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J38" s="11" t="s">
         <v>34</v>
@@ -4411,16 +4409,16 @@
         <v>26</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>31</v>
@@ -4432,7 +4430,7 @@
         <v>32</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J39" s="8" t="s">
         <v>34</v>
@@ -4446,16 +4444,16 @@
         <v>26</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F40" s="11" t="s">
         <v>31</v>
@@ -4467,7 +4465,7 @@
         <v>32</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J40" s="11" t="s">
         <v>34</v>
@@ -4481,16 +4479,16 @@
         <v>26</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F41" s="8" t="s">
         <v>31</v>
@@ -4502,7 +4500,7 @@
         <v>32</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J41" s="8" t="s">
         <v>34</v>
@@ -4516,16 +4514,16 @@
         <v>26</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F42" s="11" t="s">
         <v>31</v>
@@ -4537,7 +4535,7 @@
         <v>32</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J42" s="11" t="s">
         <v>34</v>
@@ -4551,16 +4549,16 @@
         <v>26</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F43" s="8" t="s">
         <v>31</v>
@@ -4572,7 +4570,7 @@
         <v>32</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J43" s="8" t="s">
         <v>34</v>
@@ -4586,16 +4584,16 @@
         <v>26</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F44" s="11" t="s">
         <v>31</v>
@@ -4607,7 +4605,7 @@
         <v>32</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J44" s="11" t="s">
         <v>34</v>
@@ -4621,16 +4619,16 @@
         <v>26</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>31</v>
@@ -4642,7 +4640,7 @@
         <v>32</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J45" s="8" t="s">
         <v>34</v>
@@ -4656,16 +4654,16 @@
         <v>26</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F46" s="11" t="s">
         <v>31</v>
@@ -4677,7 +4675,7 @@
         <v>32</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J46" s="11" t="s">
         <v>34</v>
@@ -4691,16 +4689,16 @@
         <v>26</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F47" s="8" t="s">
         <v>31</v>
@@ -4712,7 +4710,7 @@
         <v>32</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J47" s="8" t="s">
         <v>34</v>
@@ -4726,16 +4724,16 @@
         <v>26</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C48" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F48" s="11" t="s">
         <v>31</v>
@@ -4747,7 +4745,7 @@
         <v>32</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J48" s="11" t="s">
         <v>34</v>
@@ -4761,16 +4759,16 @@
         <v>26</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F49" s="8" t="s">
         <v>31</v>
@@ -4782,7 +4780,7 @@
         <v>32</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J49" s="8" t="s">
         <v>34</v>
@@ -4796,16 +4794,16 @@
         <v>26</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C50" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E50" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F50" s="11" t="s">
         <v>31</v>
@@ -4817,7 +4815,7 @@
         <v>32</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J50" s="11" t="s">
         <v>34</v>
@@ -4831,16 +4829,16 @@
         <v>26</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F51" s="8" t="s">
         <v>31</v>
@@ -4852,7 +4850,7 @@
         <v>32</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J51" s="8" t="s">
         <v>34</v>
@@ -4866,16 +4864,16 @@
         <v>26</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C52" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E52" s="11" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F52" s="11" t="s">
         <v>31</v>
@@ -4887,7 +4885,7 @@
         <v>32</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J52" s="11" t="s">
         <v>34</v>
@@ -4901,16 +4899,16 @@
         <v>26</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F53" s="8" t="s">
         <v>31</v>
@@ -4922,7 +4920,7 @@
         <v>32</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J53" s="8" t="s">
         <v>34</v>
@@ -4936,16 +4934,16 @@
         <v>26</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C54" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E54" s="11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F54" s="11" t="s">
         <v>31</v>
@@ -4957,7 +4955,7 @@
         <v>32</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J54" s="11" t="s">
         <v>34</v>
@@ -4971,16 +4969,16 @@
         <v>26</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F55" s="8" t="s">
         <v>31</v>
@@ -4992,7 +4990,7 @@
         <v>32</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J55" s="8" t="s">
         <v>34</v>
@@ -5006,16 +5004,16 @@
         <v>26</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C56" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F56" s="11" t="s">
         <v>31</v>
@@ -5027,7 +5025,7 @@
         <v>32</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J56" s="11" t="s">
         <v>34</v>
@@ -5041,16 +5039,16 @@
         <v>26</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F57" s="8" t="s">
         <v>31</v>
@@ -5062,7 +5060,7 @@
         <v>32</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J57" s="8" t="s">
         <v>34</v>
@@ -5076,16 +5074,16 @@
         <v>26</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C58" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E58" s="11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F58" s="11" t="s">
         <v>31</v>
@@ -5097,7 +5095,7 @@
         <v>32</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J58" s="11" t="s">
         <v>34</v>
@@ -5111,16 +5109,16 @@
         <v>26</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F59" s="8" t="s">
         <v>31</v>
@@ -5132,7 +5130,7 @@
         <v>32</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J59" s="8" t="s">
         <v>34</v>
@@ -5146,16 +5144,16 @@
         <v>26</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C60" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F60" s="11" t="s">
         <v>31</v>
@@ -5167,7 +5165,7 @@
         <v>32</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J60" s="11" t="s">
         <v>34</v>
@@ -5181,16 +5179,16 @@
         <v>26</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F61" s="8" t="s">
         <v>31</v>
@@ -5202,7 +5200,7 @@
         <v>32</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="J61" s="8" t="s">
         <v>34</v>
@@ -5216,16 +5214,16 @@
         <v>26</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C62" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>31</v>
@@ -5237,7 +5235,7 @@
         <v>32</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J62" s="11" t="s">
         <v>34</v>
@@ -5251,16 +5249,16 @@
         <v>26</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F63" s="8" t="s">
         <v>31</v>
@@ -5272,7 +5270,7 @@
         <v>32</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J63" s="8" t="s">
         <v>34</v>
@@ -5286,16 +5284,16 @@
         <v>26</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C64" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E64" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F64" s="11" t="s">
         <v>31</v>
@@ -5307,7 +5305,7 @@
         <v>32</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="J64" s="11" t="s">
         <v>34</v>
@@ -5321,16 +5319,16 @@
         <v>26</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F65" s="8" t="s">
         <v>31</v>
@@ -5342,7 +5340,7 @@
         <v>32</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J65" s="8" t="s">
         <v>34</v>
@@ -5356,16 +5354,16 @@
         <v>26</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C66" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E66" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F66" s="11" t="s">
         <v>31</v>
@@ -5377,7 +5375,7 @@
         <v>32</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J66" s="11" t="s">
         <v>34</v>
@@ -5391,28 +5389,26 @@
         <v>26</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>28</v>
+        <v>122</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F67" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="G67" s="8">
-        <v>39</v>
-      </c>
+      <c r="G67" s="8"/>
       <c r="H67" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="J67" s="8" t="s">
         <v>34</v>
@@ -5426,16 +5422,16 @@
         <v>26</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C68" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E68" s="11" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F68" s="11" t="s">
         <v>31</v>
@@ -5447,7 +5443,7 @@
         <v>32</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J68" s="11" t="s">
         <v>34</v>
@@ -5461,16 +5457,16 @@
         <v>26</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F69" s="8" t="s">
         <v>31</v>
@@ -5482,7 +5478,7 @@
         <v>32</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J69" s="8" t="s">
         <v>34</v>
@@ -5496,28 +5492,26 @@
         <v>26</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>28</v>
+        <v>122</v>
       </c>
       <c r="D70" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E70" s="11" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F70" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="G70" s="11">
-        <v>39</v>
-      </c>
+      <c r="G70" s="8"/>
       <c r="H70" s="11" t="s">
         <v>32</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="J70" s="11" t="s">
         <v>34</v>
@@ -5531,28 +5525,26 @@
         <v>26</v>
       </c>
       <c r="B71" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>28</v>
+        <v>122</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F71" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="G71" s="8">
-        <v>39</v>
-      </c>
+      <c r="G71" s="8"/>
       <c r="H71" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J71" s="8" t="s">
         <v>34</v>
@@ -5566,16 +5558,16 @@
         <v>26</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C72" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E72" s="11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F72" s="11" t="s">
         <v>31</v>
@@ -5587,7 +5579,7 @@
         <v>32</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J72" s="11" t="s">
         <v>34</v>
@@ -5601,16 +5593,16 @@
         <v>26</v>
       </c>
       <c r="B73" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F73" s="8" t="s">
         <v>31</v>
@@ -5622,7 +5614,7 @@
         <v>32</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J73" s="8" t="s">
         <v>34</v>
@@ -5636,16 +5628,16 @@
         <v>26</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C74" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D74" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E74" s="11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F74" s="11" t="s">
         <v>31</v>
@@ -5657,7 +5649,7 @@
         <v>32</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="J74" s="11" t="s">
         <v>34</v>
@@ -5671,16 +5663,16 @@
         <v>26</v>
       </c>
       <c r="B75" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F75" s="8" t="s">
         <v>31</v>
@@ -5692,7 +5684,7 @@
         <v>32</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="J75" s="8" t="s">
         <v>34</v>
@@ -5706,16 +5698,16 @@
         <v>26</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C76" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E76" s="11" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F76" s="11" t="s">
         <v>31</v>
@@ -5727,7 +5719,7 @@
         <v>32</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="J76" s="11" t="s">
         <v>34</v>
@@ -5741,16 +5733,16 @@
         <v>26</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F77" s="8" t="s">
         <v>31</v>
@@ -5762,7 +5754,7 @@
         <v>32</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J77" s="8" t="s">
         <v>34</v>
@@ -5776,16 +5768,16 @@
         <v>26</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C78" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E78" s="11" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F78" s="11" t="s">
         <v>31</v>
@@ -5797,7 +5789,7 @@
         <v>32</v>
       </c>
       <c r="I78" s="11" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J78" s="11" t="s">
         <v>34</v>
@@ -5811,16 +5803,16 @@
         <v>26</v>
       </c>
       <c r="B79" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F79" s="8" t="s">
         <v>31</v>
@@ -5832,7 +5824,7 @@
         <v>32</v>
       </c>
       <c r="I79" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J79" s="8" t="s">
         <v>34</v>
@@ -5846,16 +5838,16 @@
         <v>26</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C80" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E80" s="11" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F80" s="11" t="s">
         <v>31</v>
@@ -5867,7 +5859,7 @@
         <v>32</v>
       </c>
       <c r="I80" s="11" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J80" s="11" t="s">
         <v>34</v>
@@ -5881,16 +5873,16 @@
         <v>26</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F81" s="8" t="s">
         <v>31</v>
@@ -5902,7 +5894,7 @@
         <v>32</v>
       </c>
       <c r="I81" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J81" s="8" t="s">
         <v>34</v>
@@ -5916,16 +5908,16 @@
         <v>26</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C82" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E82" s="11" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F82" s="11" t="s">
         <v>31</v>
@@ -5937,7 +5929,7 @@
         <v>32</v>
       </c>
       <c r="I82" s="11" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J82" s="11" t="s">
         <v>34</v>
@@ -5951,16 +5943,16 @@
         <v>26</v>
       </c>
       <c r="B83" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F83" s="8" t="s">
         <v>31</v>
@@ -5972,7 +5964,7 @@
         <v>32</v>
       </c>
       <c r="I83" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J83" s="8" t="s">
         <v>34</v>
@@ -5986,16 +5978,16 @@
         <v>26</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C84" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D84" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E84" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F84" s="11" t="s">
         <v>31</v>
@@ -6007,7 +5999,7 @@
         <v>32</v>
       </c>
       <c r="I84" s="11" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J84" s="11" t="s">
         <v>34</v>
@@ -6021,16 +6013,16 @@
         <v>26</v>
       </c>
       <c r="B85" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D85" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F85" s="8" t="s">
         <v>31</v>
@@ -6042,7 +6034,7 @@
         <v>32</v>
       </c>
       <c r="I85" s="8" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J85" s="8" t="s">
         <v>34</v>
@@ -6056,16 +6048,16 @@
         <v>26</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C86" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E86" s="11" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F86" s="11" t="s">
         <v>31</v>
@@ -6077,7 +6069,7 @@
         <v>32</v>
       </c>
       <c r="I86" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J86" s="11" t="s">
         <v>34</v>
@@ -6091,16 +6083,16 @@
         <v>26</v>
       </c>
       <c r="B87" s="8" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D87" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>31</v>
@@ -6112,7 +6104,7 @@
         <v>32</v>
       </c>
       <c r="I87" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="J87" s="8" t="s">
         <v>34</v>
@@ -6126,16 +6118,16 @@
         <v>26</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C88" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E88" s="11" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F88" s="11" t="s">
         <v>31</v>
@@ -6147,7 +6139,7 @@
         <v>32</v>
       </c>
       <c r="I88" s="11" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J88" s="11" t="s">
         <v>34</v>
@@ -6161,16 +6153,16 @@
         <v>26</v>
       </c>
       <c r="B89" s="8" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>31</v>
@@ -6182,7 +6174,7 @@
         <v>32</v>
       </c>
       <c r="I89" s="8" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J89" s="8" t="s">
         <v>34</v>
@@ -6196,16 +6188,16 @@
         <v>26</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C90" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D90" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E90" s="11" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F90" s="11" t="s">
         <v>31</v>
@@ -6217,7 +6209,7 @@
         <v>32</v>
       </c>
       <c r="I90" s="11" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J90" s="11" t="s">
         <v>34</v>
@@ -6231,16 +6223,16 @@
         <v>26</v>
       </c>
       <c r="B91" s="8" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F91" s="8" t="s">
         <v>31</v>
@@ -6252,7 +6244,7 @@
         <v>32</v>
       </c>
       <c r="I91" s="8" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J91" s="8" t="s">
         <v>34</v>
@@ -6266,16 +6258,16 @@
         <v>26</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C92" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D92" s="11" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E92" s="11" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F92" s="11" t="s">
         <v>31</v>
@@ -6287,7 +6279,7 @@
         <v>32</v>
       </c>
       <c r="I92" s="11" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J92" s="11" t="s">
         <v>34</v>
@@ -6301,16 +6293,16 @@
         <v>26</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F93" s="8" t="s">
         <v>31</v>
@@ -6322,7 +6314,7 @@
         <v>32</v>
       </c>
       <c r="I93" s="8" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J93" s="8" t="s">
         <v>34</v>
@@ -6336,16 +6328,16 @@
         <v>26</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C94" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D94" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E94" s="11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F94" s="11" t="s">
         <v>31</v>
@@ -6357,7 +6349,7 @@
         <v>32</v>
       </c>
       <c r="I94" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J94" s="11" t="s">
         <v>34</v>
@@ -6371,16 +6363,16 @@
         <v>26</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C95" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D95" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E95" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F95" s="8" t="s">
         <v>31</v>
@@ -6392,7 +6384,7 @@
         <v>32</v>
       </c>
       <c r="I95" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J95" s="8" t="s">
         <v>34</v>
@@ -6406,16 +6398,16 @@
         <v>26</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C96" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D96" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E96" s="11" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F96" s="11" t="s">
         <v>31</v>
@@ -6427,7 +6419,7 @@
         <v>32</v>
       </c>
       <c r="I96" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J96" s="11" t="s">
         <v>34</v>
@@ -6441,16 +6433,16 @@
         <v>26</v>
       </c>
       <c r="B97" s="8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C97" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D97" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F97" s="8" t="s">
         <v>31</v>
@@ -6462,7 +6454,7 @@
         <v>32</v>
       </c>
       <c r="I97" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J97" s="8" t="s">
         <v>34</v>
@@ -6476,16 +6468,16 @@
         <v>26</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C98" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D98" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E98" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F98" s="11" t="s">
         <v>31</v>
@@ -6497,7 +6489,7 @@
         <v>32</v>
       </c>
       <c r="I98" s="11" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J98" s="11" t="s">
         <v>34</v>
@@ -6511,16 +6503,16 @@
         <v>26</v>
       </c>
       <c r="B99" s="8" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C99" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D99" s="8" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F99" s="8" t="s">
         <v>31</v>
@@ -6532,7 +6524,7 @@
         <v>32</v>
       </c>
       <c r="I99" s="8" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="J99" s="8" t="s">
         <v>34</v>
@@ -6546,16 +6538,16 @@
         <v>26</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C100" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D100" s="11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E100" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F100" s="11" t="s">
         <v>31</v>
@@ -6567,7 +6559,7 @@
         <v>32</v>
       </c>
       <c r="I100" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="J100" s="11" t="s">
         <v>34</v>
@@ -6581,16 +6573,16 @@
         <v>26</v>
       </c>
       <c r="B101" s="8" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C101" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D101" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F101" s="8" t="s">
         <v>31</v>
@@ -6602,7 +6594,7 @@
         <v>32</v>
       </c>
       <c r="I101" s="8" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="J101" s="8" t="s">
         <v>34</v>
@@ -6616,16 +6608,16 @@
         <v>26</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C102" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D102" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E102" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F102" s="11" t="s">
         <v>31</v>
@@ -6637,7 +6629,7 @@
         <v>32</v>
       </c>
       <c r="I102" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J102" s="11" t="s">
         <v>34</v>
@@ -6651,16 +6643,16 @@
         <v>26</v>
       </c>
       <c r="B103" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C103" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D103" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F103" s="8" t="s">
         <v>31</v>
@@ -6672,7 +6664,7 @@
         <v>32</v>
       </c>
       <c r="I103" s="8" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="J103" s="8" t="s">
         <v>34</v>
@@ -6686,16 +6678,16 @@
         <v>26</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C104" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D104" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E104" s="11" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F104" s="11" t="s">
         <v>31</v>
@@ -6707,7 +6699,7 @@
         <v>32</v>
       </c>
       <c r="I104" s="11" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J104" s="11" t="s">
         <v>34</v>
@@ -6721,16 +6713,16 @@
         <v>26</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C105" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F105" s="8" t="s">
         <v>31</v>
@@ -6742,7 +6734,7 @@
         <v>32</v>
       </c>
       <c r="I105" s="8" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J105" s="8" t="s">
         <v>34</v>
@@ -6756,16 +6748,16 @@
         <v>26</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C106" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D106" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E106" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F106" s="11" t="s">
         <v>31</v>
@@ -6777,7 +6769,7 @@
         <v>32</v>
       </c>
       <c r="I106" s="11" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J106" s="11" t="s">
         <v>34</v>
@@ -6791,16 +6783,16 @@
         <v>26</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C107" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D107" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F107" s="8" t="s">
         <v>31</v>
@@ -6812,7 +6804,7 @@
         <v>32</v>
       </c>
       <c r="I107" s="8" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="J107" s="8" t="s">
         <v>34</v>
@@ -6826,16 +6818,16 @@
         <v>26</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C108" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D108" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E108" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F108" s="11" t="s">
         <v>31</v>
@@ -6847,7 +6839,7 @@
         <v>32</v>
       </c>
       <c r="I108" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="J108" s="11" t="s">
         <v>34</v>
@@ -6861,16 +6853,16 @@
         <v>26</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C109" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E109" s="8" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F109" s="8" t="s">
         <v>31</v>
@@ -6882,7 +6874,7 @@
         <v>32</v>
       </c>
       <c r="I109" s="8" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="J109" s="8" t="s">
         <v>34</v>
@@ -6896,16 +6888,16 @@
         <v>26</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C110" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D110" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E110" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F110" s="11" t="s">
         <v>31</v>
@@ -6917,7 +6909,7 @@
         <v>32</v>
       </c>
       <c r="I110" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="J110" s="11" t="s">
         <v>34</v>
@@ -6931,16 +6923,16 @@
         <v>26</v>
       </c>
       <c r="B111" s="8" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C111" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D111" s="8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E111" s="8" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F111" s="8" t="s">
         <v>31</v>
@@ -6952,7 +6944,7 @@
         <v>32</v>
       </c>
       <c r="I111" s="8" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="J111" s="8" t="s">
         <v>34</v>
@@ -6966,19 +6958,19 @@
         <v>26</v>
       </c>
       <c r="B112" s="11" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C112" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D112" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E112" s="11" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F112" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G112" s="11">
         <v>69</v>
@@ -6987,7 +6979,7 @@
         <v>32</v>
       </c>
       <c r="I112" s="11" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="J112" s="11" t="s">
         <v>34</v>
@@ -7001,19 +6993,19 @@
         <v>26</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C113" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D113" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E113" s="8" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F113" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G113" s="8">
         <v>69</v>
@@ -7022,7 +7014,7 @@
         <v>32</v>
       </c>
       <c r="I113" s="8" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J113" s="8" t="s">
         <v>34</v>
@@ -7036,19 +7028,19 @@
         <v>26</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C114" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D114" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E114" s="11" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F114" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G114" s="11">
         <v>69</v>
@@ -7057,7 +7049,7 @@
         <v>32</v>
       </c>
       <c r="I114" s="11" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="J114" s="11" t="s">
         <v>34</v>
@@ -7071,19 +7063,19 @@
         <v>26</v>
       </c>
       <c r="B115" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C115" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D115" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E115" s="8" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F115" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G115" s="8">
         <v>69</v>
@@ -7092,7 +7084,7 @@
         <v>32</v>
       </c>
       <c r="I115" s="8" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J115" s="8" t="s">
         <v>34</v>
@@ -7106,19 +7098,19 @@
         <v>26</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C116" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D116" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E116" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F116" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G116" s="11">
         <v>69</v>
@@ -7127,7 +7119,7 @@
         <v>32</v>
       </c>
       <c r="I116" s="11" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="J116" s="11" t="s">
         <v>34</v>
@@ -7141,19 +7133,19 @@
         <v>26</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C117" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D117" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F117" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G117" s="8">
         <v>69</v>
@@ -7162,7 +7154,7 @@
         <v>32</v>
       </c>
       <c r="I117" s="8" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J117" s="8" t="s">
         <v>34</v>
@@ -7176,19 +7168,19 @@
         <v>26</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C118" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D118" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E118" s="11" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F118" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G118" s="11">
         <v>69</v>
@@ -7197,7 +7189,7 @@
         <v>32</v>
       </c>
       <c r="I118" s="11" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J118" s="11" t="s">
         <v>34</v>
@@ -7211,19 +7203,19 @@
         <v>26</v>
       </c>
       <c r="B119" s="8" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C119" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D119" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E119" s="8" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F119" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G119" s="8">
         <v>69</v>
@@ -7232,7 +7224,7 @@
         <v>32</v>
       </c>
       <c r="I119" s="8" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J119" s="8" t="s">
         <v>34</v>
@@ -7246,19 +7238,19 @@
         <v>26</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C120" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D120" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E120" s="11" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F120" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G120" s="11">
         <v>69</v>
@@ -7267,7 +7259,7 @@
         <v>32</v>
       </c>
       <c r="I120" s="11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="J120" s="11" t="s">
         <v>34</v>
@@ -7281,19 +7273,19 @@
         <v>26</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C121" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D121" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E121" s="8" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F121" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G121" s="8">
         <v>69</v>
@@ -7302,7 +7294,7 @@
         <v>32</v>
       </c>
       <c r="I121" s="8" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="J121" s="8" t="s">
         <v>34</v>
@@ -7316,19 +7308,19 @@
         <v>26</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C122" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D122" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E122" s="11" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F122" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G122" s="11">
         <v>69</v>
@@ -7337,7 +7329,7 @@
         <v>32</v>
       </c>
       <c r="I122" s="11" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="J122" s="11" t="s">
         <v>34</v>
@@ -7351,19 +7343,19 @@
         <v>26</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C123" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D123" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F123" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G123" s="8">
         <v>69</v>
@@ -7372,7 +7364,7 @@
         <v>32</v>
       </c>
       <c r="I123" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="J123" s="8" t="s">
         <v>34</v>
@@ -7386,19 +7378,19 @@
         <v>26</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C124" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D124" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E124" s="11" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F124" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G124" s="11">
         <v>69</v>
@@ -7407,7 +7399,7 @@
         <v>32</v>
       </c>
       <c r="I124" s="11" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J124" s="11" t="s">
         <v>34</v>
@@ -7421,19 +7413,19 @@
         <v>26</v>
       </c>
       <c r="B125" s="8" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C125" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D125" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E125" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F125" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G125" s="8">
         <v>69</v>
@@ -7442,7 +7434,7 @@
         <v>32</v>
       </c>
       <c r="I125" s="8" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J125" s="8" t="s">
         <v>34</v>
@@ -7456,19 +7448,19 @@
         <v>26</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C126" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D126" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E126" s="11" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F126" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G126" s="11">
         <v>69</v>
@@ -7477,7 +7469,7 @@
         <v>32</v>
       </c>
       <c r="I126" s="11" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="J126" s="11" t="s">
         <v>34</v>
@@ -7491,19 +7483,19 @@
         <v>26</v>
       </c>
       <c r="B127" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C127" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D127" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E127" s="8" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F127" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G127" s="8">
         <v>69</v>
@@ -7512,7 +7504,7 @@
         <v>32</v>
       </c>
       <c r="I127" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="J127" s="8" t="s">
         <v>34</v>
@@ -7526,19 +7518,19 @@
         <v>26</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C128" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D128" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E128" s="11" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F128" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G128" s="11">
         <v>69</v>
@@ -7547,7 +7539,7 @@
         <v>32</v>
       </c>
       <c r="I128" s="11" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J128" s="11" t="s">
         <v>34</v>
@@ -7561,19 +7553,19 @@
         <v>26</v>
       </c>
       <c r="B129" s="8" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C129" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D129" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E129" s="8" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="F129" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G129" s="8">
         <v>69</v>
@@ -7582,7 +7574,7 @@
         <v>32</v>
       </c>
       <c r="I129" s="8" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="J129" s="8" t="s">
         <v>34</v>
@@ -7596,19 +7588,19 @@
         <v>26</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C130" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D130" s="11" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E130" s="11" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F130" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G130" s="11">
         <v>69</v>
@@ -7617,7 +7609,7 @@
         <v>32</v>
       </c>
       <c r="I130" s="11" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="J130" s="11" t="s">
         <v>34</v>
@@ -7631,19 +7623,19 @@
         <v>26</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C131" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D131" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E131" s="8" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F131" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G131" s="8">
         <v>74</v>
@@ -7652,7 +7644,7 @@
         <v>32</v>
       </c>
       <c r="I131" s="8" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J131" s="8" t="s">
         <v>34</v>
@@ -7666,19 +7658,19 @@
         <v>26</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C132" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D132" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E132" s="11" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F132" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G132" s="11">
         <v>74</v>
@@ -7687,7 +7679,7 @@
         <v>32</v>
       </c>
       <c r="I132" s="11" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="J132" s="11" t="s">
         <v>34</v>
@@ -7701,19 +7693,19 @@
         <v>26</v>
       </c>
       <c r="B133" s="8" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C133" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D133" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E133" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F133" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G133" s="8">
         <v>74</v>
@@ -7722,7 +7714,7 @@
         <v>32</v>
       </c>
       <c r="I133" s="8" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J133" s="8" t="s">
         <v>34</v>
@@ -7736,19 +7728,19 @@
         <v>26</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C134" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D134" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E134" s="11" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F134" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G134" s="11">
         <v>74</v>
@@ -7757,7 +7749,7 @@
         <v>32</v>
       </c>
       <c r="I134" s="11" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J134" s="11" t="s">
         <v>34</v>
@@ -7771,19 +7763,19 @@
         <v>26</v>
       </c>
       <c r="B135" s="8" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C135" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D135" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E135" s="8" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F135" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G135" s="8">
         <v>74</v>
@@ -7792,7 +7784,7 @@
         <v>32</v>
       </c>
       <c r="I135" s="8" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="J135" s="8" t="s">
         <v>34</v>
@@ -7806,19 +7798,19 @@
         <v>26</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C136" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D136" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E136" s="11" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F136" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G136" s="11">
         <v>74</v>
@@ -7827,7 +7819,7 @@
         <v>32</v>
       </c>
       <c r="I136" s="11" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J136" s="11" t="s">
         <v>34</v>
@@ -7841,19 +7833,19 @@
         <v>26</v>
       </c>
       <c r="B137" s="8" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C137" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D137" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E137" s="8" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F137" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G137" s="8">
         <v>74</v>
@@ -7862,7 +7854,7 @@
         <v>32</v>
       </c>
       <c r="I137" s="8" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J137" s="8" t="s">
         <v>34</v>
@@ -7876,19 +7868,19 @@
         <v>26</v>
       </c>
       <c r="B138" s="11" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C138" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D138" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E138" s="11" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F138" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G138" s="11">
         <v>74</v>
@@ -7897,7 +7889,7 @@
         <v>32</v>
       </c>
       <c r="I138" s="11" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J138" s="11" t="s">
         <v>34</v>
@@ -7911,19 +7903,19 @@
         <v>26</v>
       </c>
       <c r="B139" s="8" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C139" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D139" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E139" s="8" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F139" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G139" s="8">
         <v>74</v>
@@ -7932,7 +7924,7 @@
         <v>32</v>
       </c>
       <c r="I139" s="8" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J139" s="8" t="s">
         <v>34</v>
@@ -7946,19 +7938,19 @@
         <v>26</v>
       </c>
       <c r="B140" s="11" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C140" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D140" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E140" s="11" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F140" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G140" s="11">
         <v>74</v>
@@ -7967,7 +7959,7 @@
         <v>32</v>
       </c>
       <c r="I140" s="11" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="J140" s="11" t="s">
         <v>34</v>
@@ -7981,19 +7973,19 @@
         <v>26</v>
       </c>
       <c r="B141" s="8" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C141" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D141" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E141" s="8" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F141" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G141" s="8">
         <v>74</v>
@@ -8002,7 +7994,7 @@
         <v>32</v>
       </c>
       <c r="I141" s="8" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J141" s="8" t="s">
         <v>34</v>
@@ -8016,19 +8008,19 @@
         <v>26</v>
       </c>
       <c r="B142" s="11" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C142" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D142" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E142" s="11" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F142" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G142" s="11">
         <v>74</v>
@@ -8037,7 +8029,7 @@
         <v>32</v>
       </c>
       <c r="I142" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="J142" s="11" t="s">
         <v>34</v>
@@ -8051,19 +8043,19 @@
         <v>26</v>
       </c>
       <c r="B143" s="8" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C143" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D143" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E143" s="8" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F143" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G143" s="8">
         <v>74</v>
@@ -8072,7 +8064,7 @@
         <v>32</v>
       </c>
       <c r="I143" s="8" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J143" s="8" t="s">
         <v>34</v>
@@ -8086,19 +8078,19 @@
         <v>26</v>
       </c>
       <c r="B144" s="11" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C144" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D144" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E144" s="11" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F144" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G144" s="11">
         <v>74</v>
@@ -8107,7 +8099,7 @@
         <v>32</v>
       </c>
       <c r="I144" s="11" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="J144" s="11" t="s">
         <v>34</v>
@@ -8121,19 +8113,19 @@
         <v>26</v>
       </c>
       <c r="B145" s="8" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C145" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D145" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E145" s="8" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F145" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G145" s="8">
         <v>74</v>
@@ -8142,7 +8134,7 @@
         <v>32</v>
       </c>
       <c r="I145" s="8" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J145" s="8" t="s">
         <v>34</v>
@@ -8156,19 +8148,19 @@
         <v>26</v>
       </c>
       <c r="B146" s="11" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C146" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D146" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E146" s="11" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F146" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G146" s="11">
         <v>74</v>
@@ -8177,7 +8169,7 @@
         <v>32</v>
       </c>
       <c r="I146" s="11" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="J146" s="11" t="s">
         <v>34</v>
@@ -8191,19 +8183,19 @@
         <v>26</v>
       </c>
       <c r="B147" s="8" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C147" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D147" s="8" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E147" s="8" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F147" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G147" s="8">
         <v>74</v>
@@ -8212,7 +8204,7 @@
         <v>32</v>
       </c>
       <c r="I147" s="8" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J147" s="8" t="s">
         <v>34</v>
@@ -8226,19 +8218,19 @@
         <v>26</v>
       </c>
       <c r="B148" s="11" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="C148" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D148" s="11" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E148" s="11" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F148" s="11" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G148" s="11">
         <v>74</v>
@@ -8247,7 +8239,7 @@
         <v>32</v>
       </c>
       <c r="I148" s="11" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J148" s="11" t="s">
         <v>34</v>
@@ -8261,10 +8253,10 @@
         <v>26</v>
       </c>
       <c r="B149" s="8" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D149" s="8" t="s">
         <v>486</v>
@@ -8297,7 +8289,7 @@
         <v>490</v>
       </c>
       <c r="C150" s="11" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D150" s="11" t="s">
         <v>486</v>
@@ -8330,7 +8322,7 @@
         <v>493</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D151" s="8" t="s">
         <v>486</v>
@@ -8363,7 +8355,7 @@
         <v>496</v>
       </c>
       <c r="C152" s="11" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D152" s="11" t="s">
         <v>486</v>
@@ -8396,7 +8388,7 @@
         <v>499</v>
       </c>
       <c r="C153" s="8" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D153" s="8" t="s">
         <v>486</v>
@@ -8429,7 +8421,7 @@
         <v>502</v>
       </c>
       <c r="C154" s="11" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D154" s="11" t="s">
         <v>486</v>
@@ -8462,7 +8454,7 @@
         <v>505</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D155" s="8" t="s">
         <v>486</v>
@@ -8495,7 +8487,7 @@
         <v>508</v>
       </c>
       <c r="C156" s="11" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D156" s="11" t="s">
         <v>486</v>
@@ -8528,7 +8520,7 @@
         <v>511</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D157" s="8" t="s">
         <v>486</v>
@@ -8561,7 +8553,7 @@
         <v>514</v>
       </c>
       <c r="C158" s="11" t="s">
-        <v>485</v>
+        <v>122</v>
       </c>
       <c r="D158" s="11" t="s">
         <v>486</v>

</xml_diff>